<commit_message>
Sensitivity structure: tornado + two-way, E1 floored at 0.0 (LA untargeted downside)
Tornado ranges trace to assumptions-log IDs; E1's floor models the LA
natural experiment directly instead of footnoting it -- the zero bar IS
the untargeted scenario, per the log's 'targeting is a design
requirement' finding. Two-way grid gains an E1=0.0 row for the same
reason; grid ships static from the script and is rebuilt as a live
Excel Data Table in the hand-finished workbook.

Filename split: script now writes model_skeleton.xlsx (gitignored,
regenerable); sidewalk_capital_model.xlsx is the canonical hand-
finished copy the script never touches.

Finding worth recording: with corrected ranges the tornado still
contradicts the spec's prediction -- cost-per-location-mitigated
(21.6M swing) dominates E1 effectiveness (5.7M), and no single
variable at its favorable extreme turns Option B positive. The
biggest lever is unit cost, not program effectiveness.
</commit_message>
<xml_diff>
--- a/03-model/sidewalk_capital_model.xlsx
+++ b/03-model/sidewalk_capital_model.xlsx
@@ -1982,12 +1982,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NPV, mitigation at scale (B) vs do nothing</t>
-        </is>
-      </c>
-      <c r="B2">
-        <f>NPV!$O$1</f>
-        <v/>
+          <t>NPV Option B vs do-nothing (Python base = NPV tab)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>-11019978</v>
       </c>
     </row>
     <row r="3">
@@ -2073,14 +2072,343 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Hand-build: tornado on every ESTIMATE input (spec rule #1), two-way on top 2 drivers.</t>
-        </is>
+          <t>TORNADO (Python-computed; ranges trace to assumptions-log IDs; E1 floored at 0.0 per LA natural experiment)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Low NPV_B</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>High NPV_B</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Swing</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Base NPV_B</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Range rationale</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Cost per location mitigated</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>-3807019</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-25445896</v>
+      </c>
+      <c r="D4" t="n">
+        <v>21638877</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-11019978</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>E1b ESTIMATE anchored to B5 ramping-crew cost; log rule: every ESTIMATE stays in the tornado</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Option B rollout share</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>-5509989</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-16529967</v>
+      </c>
+      <c r="D5" t="n">
+        <v>11019978</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-11019978</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>policy lever, not uncertainty - shown for completeness; scenario axis in the memo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>E1 mitigation effectiveness</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>-14425918</v>
+      </c>
+      <c r="C6" t="n">
+        <v>-8749352</v>
+      </c>
+      <c r="D6" t="n">
+        <v>5676566</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-11019978</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>floor 0.0 = LA untargeted downside (E1 evidence base); 0.50 targeted upper remains a guess</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Horizon (years)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>-12797701</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-8163706</v>
+      </c>
+      <c r="D7" t="n">
+        <v>4633995</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-11019978</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>F2; vs B9 50-75yr useful life</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Baseline annual claims</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>-11701166</v>
+      </c>
+      <c r="C8" t="n">
+        <v>-10475028</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1226138</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-11019978</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>L1 2015-21 avg to L3 FY23 high</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Discount rate</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>-11103934</v>
+      </c>
+      <c r="C9" t="n">
+        <v>-10634790</v>
+      </c>
+      <c r="D9" t="n">
+        <v>469145</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-11019978</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>F1 regime flux: A-94 Appendix C ~2% to reinstated 7% base</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TWO-WAY: NPV_B by E1 (rows) x $/location (cols). Rebuild as a live Excel Data Table in the hand-finished workbook (What-If Analysis; corner ='NPV'!O1, row input INPUTS!B11, col input INPUTS!B10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>E1 \ $loc</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>150</v>
+      </c>
+      <c r="C13" t="n">
+        <v>250</v>
+      </c>
+      <c r="D13" t="n">
+        <v>350</v>
+      </c>
+      <c r="E13" t="n">
+        <v>450</v>
+      </c>
+      <c r="F13" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>0</v>
+      </c>
+      <c r="B14" t="n">
+        <v>-7212959</v>
+      </c>
+      <c r="C14" t="n">
+        <v>-12021598</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-16830238</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-21638877</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-28851836</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B15" t="n">
+        <v>-6077646</v>
+      </c>
+      <c r="C15" t="n">
+        <v>-10886285</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-15694924</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-20503564</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-27716523</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="B16" t="n">
+        <v>-4942332</v>
+      </c>
+      <c r="C16" t="n">
+        <v>-9750972</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-14559611</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-19368250</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-26581209</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="B17" t="n">
+        <v>-3807019</v>
+      </c>
+      <c r="C17" t="n">
+        <v>-8615659</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-13424298</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-18232937</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-25445896</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="B18" t="n">
+        <v>-2671706</v>
+      </c>
+      <c r="C18" t="n">
+        <v>-7480345</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-12288985</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-17097624</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-24310583</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B19" t="n">
+        <v>-1536393</v>
+      </c>
+      <c r="C19" t="n">
+        <v>-6345032</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-11153671</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-15962311</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-23175270</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Business case memo: the folk liability argument fails, and here's the bar the honest case must clear
Memo written against OUTPUT-tab figures only, per spec rule: B -11.0M,
C -116.8M, breakeven ~71/location, 1.29M/yr additional benefit to
break even (Option C python mirror + derived headlines added to OUTPUT
so every memo figure has a legal source). Core argument: don't fund on
avoided-lawsuits economics -- LA spent ~226M and settlements rose --
but the case FOR investment is quantifiable: clear the 1.29M/yr bar
with ADA/asset-preservation/societal benefit lines, hit unit cost
under breakeven, and target by claims density (5 ZIPs = 45%% of
claims). README rewritten answer-first: finding in the blockquote,
start-here link to the memo, WIP banner retired.
</commit_message>
<xml_diff>
--- a/03-model/sidewalk_capital_model.xlsx
+++ b/03-model/sidewalk_capital_model.xlsx
@@ -1961,7 +1961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -2018,6 +2018,36 @@
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NPV Option C vs do-nothing (Python base, mirrors NPV tab)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>-116845288</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Breakeven cost/location for B (derived, linear in costloc)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Additional annual benefit needed for B to break even (beyond avoided claims)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1291878</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Refine sensitivity grid into a live two-variable Data Table
The E1 x cost-per-location grid was a static Python-computed block; it is
now a genuine Excel two-variable Data Table (Data > What-If Analysis):
corner cell = NPV!O1, row input = INPUTS!B11 (cost/location), column
input = INPUTS!B10 (E1 effectiveness). Editing any INPUTS driver now
recomputes the whole grid live. Values verified against the prior static
computation (all corners match); SENSITIVITY note updated to describe
the live table rather than flag it as a TODO.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WtP6zzYG9N7zKmBNu2rkNF
</commit_message>
<xml_diff>
--- a/03-model/sidewalk_capital_model.xlsx
+++ b/03-model/sidewalk_capital_model.xlsx
@@ -2295,15 +2295,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TWO-WAY: NPV_B by E1 (rows) x $/location (cols). Rebuild as a live Excel Data Table in the hand-finished workbook (What-If Analysis; corner ='NPV'!O1, row input INPUTS!B11, col input INPUTS!B10).</t>
+          <t>TWO-WAY: NPV_B by E1 (rows) x $/location (cols). Live Excel Data Table (Data -&gt; What-If Analysis): corner =NPV!O1, row input INPUTS!B11, col input INPUTS!B10 - edit any INPUTS value and this grid recalculates.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>E1 \ $loc</t>
-        </is>
+      <c r="A13">
+        <f>NPV!$O$1</f>
+        <v>-11019978</v>
       </c>
       <c r="B13" t="n">
         <v>150</v>
@@ -2325,7 +2324,8 @@
       <c r="A14" t="n">
         <v>0</v>
       </c>
-      <c r="B14" t="n">
+      <c r="B14">
+        <f t="dataTable" ref="B14:F19" dt2D="1" dtr="0" r1="INPUTS!$B$11" r2="INPUTS!$B$10" ca="1"/>
         <v>-7212959</v>
       </c>
       <c r="C14" t="n">

</xml_diff>